<commit_message>
Rerouting table: correct the indicative amounts per line
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PdcnbvMxTN9eaMqR4tfx6H
</commit_message>
<xml_diff>
--- a/output/Rerouting_Internal_to_DOH.xlsx
+++ b/output/Rerouting_Internal_to_DOH.xlsx
@@ -571,8 +571,10 @@
           <t>CONFIRMED (ruling)</t>
         </is>
       </c>
-      <c r="J2" s="3" t="n">
-        <v>728918.6100000001</v>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 682)</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -619,8 +621,10 @@
           <t>CONFIRMED (ruling)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n">
-        <v>5638.57</v>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 570)</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -667,8 +671,10 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
-        <v>728918.6100000001</v>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 2,338)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -715,8 +721,10 @@
           <t>CONFIRMED (ruling)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="n">
-        <v>32942.25</v>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 52,796)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -764,7 +772,7 @@
         </is>
       </c>
       <c r="J6" s="3" t="n">
-        <v>33803</v>
+        <v>195736.9488286315</v>
       </c>
     </row>
     <row r="7">
@@ -811,7 +819,9 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="n">
+        <v>54224.25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -857,8 +867,10 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J8" s="3" t="n">
-        <v>5638.57</v>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 17,572)</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -905,8 +917,10 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J9" s="3" t="n">
-        <v>212405.05</v>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 6,169)</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -953,8 +967,10 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J10" s="3" t="n">
-        <v>96385.54000000002</v>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>see monthly stock movement (Jan: 5,583)</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1001,9 +1017,7 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J11" s="3" t="n">
-        <v>3045</v>
-      </c>
+      <c r="J11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1530,7 +1544,7 @@
         </is>
       </c>
       <c r="J22" s="3" t="n">
-        <v>74728.05</v>
+        <v>21197.95</v>
       </c>
     </row>
     <row r="23">
@@ -1578,7 +1592,7 @@
         </is>
       </c>
       <c r="J23" s="3" t="n">
-        <v>125589.17</v>
+        <v>70487.25</v>
       </c>
     </row>
     <row r="24">
@@ -1626,7 +1640,7 @@
         </is>
       </c>
       <c r="J24" s="3" t="n">
-        <v>125589.17</v>
+        <v>70487.25</v>
       </c>
     </row>
     <row r="25">
@@ -1674,7 +1688,7 @@
         </is>
       </c>
       <c r="J25" s="3" t="n">
-        <v>1763162.330000001</v>
+        <v>181346.3900000004</v>
       </c>
     </row>
     <row r="26">
@@ -1722,7 +1736,7 @@
         </is>
       </c>
       <c r="J26" s="3" t="n">
-        <v>2394963.42</v>
+        <v>62148.42</v>
       </c>
     </row>
     <row r="27">
@@ -1770,7 +1784,7 @@
         </is>
       </c>
       <c r="J27" s="3" t="n">
-        <v>35473.23</v>
+        <v>32231.23</v>
       </c>
     </row>
     <row r="28">
@@ -1866,7 +1880,7 @@
         </is>
       </c>
       <c r="J29" s="3" t="n">
-        <v>125589.17</v>
+        <v>111874.02</v>
       </c>
     </row>
     <row r="30">
@@ -1914,7 +1928,7 @@
         </is>
       </c>
       <c r="J30" s="3" t="n">
-        <v>1763162.330000001</v>
+        <v>1581815.94</v>
       </c>
     </row>
     <row r="31">
@@ -2529,7 +2543,9 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="n">
+        <v>5638.57</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2575,7 +2591,9 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="n">
+        <v>33803</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2715,7 +2733,9 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="n">
+        <v>126679.42</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2761,7 +2781,9 @@
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="J48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="n">
+        <v>30297.55</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">

</xml_diff>